<commit_message>
Daily 15-minute brief: one story per event, top 3 per section, Model Watch
- Group the same story from different sources (shared rare key words and
  product versions, 72 h window); rank by coverage, official source, recency
- Today page: top 3 overall, then top 3 per section, never a story twice;
  reading-time meter, trending words, "also covered by" per story
- Summaries from the article's own opening sentences (no AI); bios, adverts
  and newsletter housekeeping skipped, page description used instead
- New sources: Anthropic (scraped), Anthropic Engineering and Research,
  Thoughtworks, IEA (via Google News), Green Software Foundation, and an
  Engineering Blogs section (Netflix, Meta, Stripe, Spotify and others)
- Model Watch: model news, new models on OpenRouter, trending on Hugging Face
- A failing source keeps its last good items; caches kept between runs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tech-Pulse-Sources.xlsx
+++ b/Tech-Pulse-Sources.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$4:$I$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$4:$I$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Paper venues'!$A$4:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How to use: in the yellow 'Include?' column, choose Yes or No for each source. Add your own sources at the bottom (any site with an RSS feed, or any YouTube channel). Every feed was tested on 27 Oct 2026.</t>
+          <t>How to use: in the yellow 'Include?' column, choose Yes or No for each source. Add your own sources at the bottom (any site with an RSS feed, or any YouTube channel). Every feed was tested on 28 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -625,22 +625,22 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>The Verge</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Consumer tech, gadgets, platforms, policy</t>
+          <t>Google's own announcements (The Keyword)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -652,11 +652,11 @@
         <v>46322</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/rss/index.xml</t>
+          <t>https://blog.google/rss/</t>
         </is>
       </c>
     </row>
@@ -668,22 +668,22 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Startups, funding, venture capital, product launches</t>
+          <t>Microsoft corporate announcements</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -695,11 +695,11 @@
         <v>46322</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/feed/</t>
+          <t>https://blogs.microsoft.com/feed/</t>
         </is>
       </c>
     </row>
@@ -711,22 +711,22 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Ars Technica</t>
+          <t>Apple Newsroom</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>In-depth tech, science, IT and policy</t>
+          <t>Apple press releases</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -735,14 +735,14 @@
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>https://feeds.arstechnica.com/arstechnica/index</t>
+          <t>https://www.apple.com/newsroom/rss-feed.rss</t>
         </is>
       </c>
     </row>
@@ -754,22 +754,22 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Wired</t>
+          <t>AWS News</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Tech culture, business, science, security</t>
+          <t>New AWS services and launches</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -778,14 +778,14 @@
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>https://www.wired.com/feed/rss</t>
+          <t>https://aws.amazon.com/blogs/aws/feed/</t>
         </is>
       </c>
     </row>
@@ -797,22 +797,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Engadget</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Gadgets, gaming, consumer electronics</t>
+          <t>GPUs, AI computing, data centres</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -824,11 +824,11 @@
         <v>46322</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>https://www.engadget.com/rss.xml</t>
+          <t>https://blogs.nvidia.com/feed/</t>
         </is>
       </c>
     </row>
@@ -840,22 +840,22 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>The Register</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Enterprise IT, cloud, sysadmin, chips (UK)</t>
+          <t>OpenAI model releases, research, product news</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -867,11 +867,11 @@
         <v>46322</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>https://www.theregister.com/headlines.atom</t>
+          <t>https://openai.com/news/rss.xml</t>
         </is>
       </c>
     </row>
@@ -883,22 +883,22 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>MIT Technology Review</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company site (scraped, no feed)</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Emerging tech, AI, biotech, climate tech</t>
+          <t>Anthropic announcements: Claude models, products, policy</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -910,11 +910,11 @@
         <v>46322</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>https://www.technologyreview.com/feed/</t>
+          <t>https://www.anthropic.com/news</t>
         </is>
       </c>
     </row>
@@ -926,22 +926,22 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Techmeme</t>
+          <t>Google DeepMind</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Aggregator</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>The day's top tech stories from across the web</t>
+          <t>DeepMind research and model releases</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -953,11 +953,11 @@
         <v>46322</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>https://www.techmeme.com/feed.xml</t>
+          <t>https://deepmind.google/blog/rss.xml</t>
         </is>
       </c>
     </row>
@@ -969,22 +969,22 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Hacker News (150+ pts)</t>
+          <t>Samsung Newsroom</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Aggregator</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Popular Hacker News links (150+ points only)</t>
+          <t>Samsung devices, chips, press releases</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -996,11 +996,11 @@
         <v>46322</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>https://hnrss.org/frontpage?points=150</t>
+          <t>https://news.samsung.com/global/feed</t>
         </is>
       </c>
     </row>
@@ -1012,22 +1012,22 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Rest of World</t>
+          <t>Thoughtworks</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Tech outside the US and Europe (Asia, Africa, LatAm)</t>
+          <t>Thoughtworks insights: AI in delivery, architecture, tech strategy</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1039,11 +1039,11 @@
         <v>46321</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>https://restofworld.org/feed/latest</t>
+          <t>https://www.thoughtworks.com/rss/insights.xml</t>
         </is>
       </c>
     </row>
@@ -1055,22 +1055,22 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Model Watch</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>The Next Web</t>
+          <t>Hugging Face</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>European tech, startups, deep tech</t>
+          <t>Open models, datasets, tooling tutorials</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1082,11 +1082,11 @@
         <v>46322</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>https://thenextweb.com/feed</t>
+          <t>https://huggingface.co/blog/feed.xml</t>
         </is>
       </c>
     </row>
@@ -1098,22 +1098,22 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Model Watch</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>9to5Mac</t>
+          <t>Qwen</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official lab blog</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Apple, iPhone, Mac (high volume)</t>
+          <t>Alibaba's Qwen model releases</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1122,14 +1122,14 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>46322</v>
+        <v>45922</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>https://9to5mac.com/feed/</t>
+          <t>https://qwenlm.github.io/blog/index.xml</t>
         </is>
       </c>
     </row>
@@ -1141,22 +1141,22 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>9to5Google</t>
+          <t>Anthropic Engineering</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company site (scraped, no feed)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Google, Android, Pixel (high volume)</t>
+          <t>How Anthropic builds agents, Claude Code and its infrastructure</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1165,14 +1165,14 @@
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>46322</v>
+        <v>46308</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>https://9to5google.com/feed/</t>
+          <t>https://www.anthropic.com/engineering</t>
         </is>
       </c>
     </row>
@@ -1184,22 +1184,22 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Anthropic Research</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Official company site (scraped, no feed)</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Google's own announcements (The Keyword)</t>
+          <t>Anthropic research: alignment, interpretability, AI and the economy</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1211,11 +1211,11 @@
         <v>46322</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>https://blog.google/rss/</t>
+          <t>https://www.anthropic.com/research</t>
         </is>
       </c>
     </row>
@@ -1227,22 +1227,22 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Simon Willison</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Expert blog</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Microsoft corporate announcements</t>
+          <t>Daily hands-on notes on LLMs and AI tools</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1251,14 +1251,14 @@
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>https://blogs.microsoft.com/feed/</t>
+          <t>https://simonwillison.net/atom/everything/</t>
         </is>
       </c>
     </row>
@@ -1270,22 +1270,22 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Apple Newsroom</t>
+          <t>Latent Space</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Newsletter / podcast</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Apple press releases</t>
+          <t>AI engineering, agents, interviews with builders</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1297,11 +1297,11 @@
         <v>46322</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>https://www.apple.com/newsroom/rss-feed.rss</t>
+          <t>https://www.latent.space/feed</t>
         </is>
       </c>
     </row>
@@ -1313,22 +1313,22 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Meta Engineering</t>
+          <t>Import AI</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Newsletter</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Meta engineering: infra, AI, open source</t>
+          <t>Jack Clark's weekly AI research and policy digest</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>https://engineering.fb.com/feed/</t>
+          <t>https://importai.substack.com/feed</t>
         </is>
       </c>
     </row>
@@ -1356,22 +1356,22 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>AWS News</t>
+          <t>Interconnects</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Newsletter</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>New AWS services and launches</t>
+          <t>Nathan Lambert on open models, RLHF, post-training</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1380,14 +1380,14 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>https://aws.amazon.com/blogs/aws/feed/</t>
+          <t>https://www.interconnects.ai/feed</t>
         </is>
       </c>
     </row>
@@ -1399,22 +1399,22 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Ahead of AI</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Newsletter</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>GPUs, AI computing, data centres</t>
+          <t>Sebastian Raschka on LLM research papers</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1423,14 +1423,14 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>https://blogs.nvidia.com/feed/</t>
+          <t>https://magazine.sebastianraschka.com/feed</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google Research</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Research lab blog</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>OpenAI model releases, research, product news</t>
+          <t>Google Research papers explained</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1466,14 +1466,14 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>https://openai.com/news/rss.xml</t>
+          <t>https://research.google/blog/rss/</t>
         </is>
       </c>
     </row>
@@ -1485,22 +1485,22 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Google DeepMind</t>
+          <t>Microsoft Research</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Research lab blog</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>DeepMind research and model releases</t>
+          <t>Microsoft Research news and papers</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1512,11 +1512,11 @@
         <v>46317</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>https://deepmind.google/blog/rss.xml</t>
+          <t>https://www.microsoft.com/en-us/research/feed/</t>
         </is>
       </c>
     </row>
@@ -1528,22 +1528,22 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Samsung Newsroom</t>
+          <t>BAIR Blog</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Research lab blog</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Samsung devices, chips, press releases</t>
+          <t>Berkeley AI Research (posts rarely)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1552,14 +1552,14 @@
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>46322</v>
+        <v>46232</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/global/feed</t>
+          <t>https://bair.berkeley.edu/blog/feed.xml</t>
         </is>
       </c>
     </row>
@@ -1571,22 +1571,22 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Netflix Tech Blog</t>
+          <t>The Decoder</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Large-scale engineering at Netflix</t>
+          <t>Daily AI news</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1595,14 +1595,14 @@
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>https://netflixtechblog.com/feed</t>
+          <t>https://the-decoder.com/feed/</t>
         </is>
       </c>
     </row>
@@ -1614,22 +1614,22 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>AI &amp; Agents</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>MarkTechPost</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Networking, security, edge computing, AI infra</t>
+          <t>AI research news and paper summaries</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1645,14 +1645,14 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>https://blog.cloudflare.com/rss/</t>
+          <t>https://www.marktechpost.com/feed/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1662,33 +1662,29 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Hugging Face</t>
+          <t>VentureBeat AI</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Open models, datasets, tooling tutorials</t>
+          <t>Enterprise AI business news</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>8</v>
-      </c>
+          <t>No: feed is broken</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="5" t="n"/>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>https://huggingface.co/blog/feed.xml</t>
+          <t>https://venturebeat.com/category/ai/feed/</t>
         </is>
       </c>
     </row>
@@ -1700,22 +1696,22 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Simon Willison</t>
+          <t>InfoQ</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Expert blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Daily hands-on notes on LLMs and AI tools</t>
+          <t>Software architecture, DevOps, practices, conference talks</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1724,14 +1720,14 @@
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>https://simonwillison.net/atom/everything/</t>
+          <t>https://feed.infoq.com/</t>
         </is>
       </c>
     </row>
@@ -1743,22 +1739,22 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Latent Space</t>
+          <t>Martin Fowler</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Newsletter / podcast</t>
+          <t>Expert blog</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>AI engineering, agents, interviews with builders</t>
+          <t>Software design, refactoring, architecture</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1767,14 +1763,14 @@
         </is>
       </c>
       <c r="G31" s="7" t="n">
-        <v>46322</v>
+        <v>46316</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>https://www.latent.space/feed</t>
+          <t>https://martinfowler.com/feed.atom</t>
         </is>
       </c>
     </row>
@@ -1786,12 +1782,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Import AI</t>
+          <t>The Pragmatic Engineer</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -1801,7 +1797,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Jack Clark's weekly AI research and policy digest</t>
+          <t>Gergely Orosz on the software industry and teams</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -1810,14 +1806,14 @@
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>https://importai.substack.com/feed</t>
+          <t>https://newsletter.pragmaticengineer.com/feed</t>
         </is>
       </c>
     </row>
@@ -1829,22 +1825,22 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Interconnects</t>
+          <t>GitHub Blog</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Newsletter</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Nathan Lambert on open models, RLHF, post-training</t>
+          <t>GitHub, Copilot, open source, dev tooling</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -1853,14 +1849,14 @@
         </is>
       </c>
       <c r="G33" s="7" t="n">
-        <v>46320</v>
+        <v>46317</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>2</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>https://www.interconnects.ai/feed</t>
+          <t>https://github.blog/feed/</t>
         </is>
       </c>
     </row>
@@ -1872,22 +1868,22 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Ahead of AI</t>
+          <t>Stack Overflow Blog</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Newsletter</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Sebastian Raschka on LLM research papers</t>
+          <t>Developer trends, surveys, engineering</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -1896,14 +1892,14 @@
         </is>
       </c>
       <c r="G34" s="7" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>https://magazine.sebastianraschka.com/feed</t>
+          <t>https://stackoverflow.blog/feed/</t>
         </is>
       </c>
     </row>
@@ -1915,22 +1911,22 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Google Research</t>
+          <t>IEEE Spectrum Computing</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Research lab blog</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Google Research papers explained</t>
+          <t>IEEE coverage of computing and software</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -1939,14 +1935,14 @@
         </is>
       </c>
       <c r="G35" s="7" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>https://research.google/blog/rss/</t>
+          <t>https://spectrum.ieee.org/feeds/topic/computing.rss</t>
         </is>
       </c>
     </row>
@@ -1958,22 +1954,22 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Research</t>
+          <t>LWN.net</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Research lab blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Microsoft Research news and papers</t>
+          <t>Linux kernel and open-source development</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -1982,57 +1978,53 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>46317</v>
+        <v>46322</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>https://www.microsoft.com/en-us/research/feed/</t>
+          <t>https://lwn.net/headlines/rss</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>BAIR Blog</t>
+          <t>Google for Developers</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Research lab blog</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Berkeley AI Research (posts rarely)</t>
+          <t>Gemini API, Android, Chrome and Google developer tools</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>46232</v>
-      </c>
-      <c r="H37" s="5" t="n">
-        <v>0</v>
-      </c>
+          <t>No: feed is broken</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="5" t="n"/>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>https://bair.berkeley.edu/blog/feed.xml</t>
+          <t>https://developers.googleblog.com/feeds/posts/default</t>
         </is>
       </c>
     </row>
@@ -2044,22 +2036,22 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>The Decoder</t>
+          <t>Netflix Tech Blog</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Daily AI news</t>
+          <t>Large-scale engineering at Netflix</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -2068,14 +2060,14 @@
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>https://the-decoder.com/feed/</t>
+          <t>https://netflixtechblog.com/feed</t>
         </is>
       </c>
     </row>
@@ -2087,22 +2079,22 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>MarkTechPost</t>
+          <t>Meta Engineering</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>AI research news and paper summaries</t>
+          <t>Meta engineering: infra, AI, open source</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2114,11 +2106,11 @@
         <v>46322</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>https://www.marktechpost.com/feed/</t>
+          <t>https://engineering.fb.com/feed/</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2122,22 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>AI &amp; Agents</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>VentureBeat AI</t>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Enterprise AI business news</t>
+          <t>Networking, security, edge computing, AI infra</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -2154,14 +2146,14 @@
         </is>
       </c>
       <c r="G40" s="7" t="n">
-        <v>46261</v>
+        <v>46322</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>https://venturebeat.com/category/ai/feed/</t>
+          <t>https://blog.cloudflare.com/rss/</t>
         </is>
       </c>
     </row>
@@ -2173,22 +2165,22 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>InfoQ</t>
+          <t>Airbnb Engineering</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Software architecture, DevOps, practices, conference talks</t>
+          <t>Search, ML and infrastructure at Airbnb</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -2197,14 +2189,14 @@
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>46322</v>
+        <v>46308</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>https://feed.infoq.com/</t>
+          <t>https://medium.com/feed/airbnb-engineering</t>
         </is>
       </c>
     </row>
@@ -2216,22 +2208,22 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Martin Fowler</t>
+          <t>Spotify Engineering</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Expert blog</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Software design, refactoring, architecture</t>
+          <t>Recommendation systems and platform engineering at Spotify</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -2240,14 +2232,14 @@
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>https://martinfowler.com/feed.atom</t>
+          <t>https://engineering.atspotify.com/feed/</t>
         </is>
       </c>
     </row>
@@ -2259,22 +2251,22 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>The Pragmatic Engineer</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Newsletter</t>
+          <t>Official company blog</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Gergely Orosz on the software industry and teams</t>
+          <t>Payments infrastructure and Stripe engineering</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -2283,14 +2275,14 @@
         </is>
       </c>
       <c r="G43" s="7" t="n">
-        <v>46317</v>
+        <v>46322</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>https://newsletter.pragmaticengineer.com/feed</t>
+          <t>https://stripe.com/blog/feed.rss</t>
         </is>
       </c>
     </row>
@@ -2302,22 +2294,22 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>GitHub Blog</t>
+          <t>Slack Engineering</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>GitHub, Copilot, open source, dev tooling</t>
+          <t>Slack's infrastructure and developer tooling</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -2326,14 +2318,14 @@
         </is>
       </c>
       <c r="G44" s="7" t="n">
-        <v>46317</v>
+        <v>46217</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>https://github.blog/feed/</t>
+          <t>https://slack.engineering/feed/</t>
         </is>
       </c>
     </row>
@@ -2345,22 +2337,22 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Stack Overflow Blog</t>
+          <t>Dropbox Tech</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Official company blog</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Developer trends, surveys, engineering</t>
+          <t>Storage, infrastructure and AI at Dropbox</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -2369,14 +2361,14 @@
         </is>
       </c>
       <c r="G45" s="7" t="n">
-        <v>46322</v>
+        <v>46294</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>https://stackoverflow.blog/feed/</t>
+          <t>https://dropbox.tech/feed</t>
         </is>
       </c>
     </row>
@@ -2388,22 +2380,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>IEEE Spectrum Computing</t>
+          <t>Pinterest Engineering</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>IEEE coverage of computing and software</t>
+          <t>ML, data and infrastructure at Pinterest</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -2412,14 +2404,14 @@
         </is>
       </c>
       <c r="G46" s="7" t="n">
-        <v>46320</v>
+        <v>46314</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>https://spectrum.ieee.org/feeds/topic/computing.rss</t>
+          <t>https://medium.com/feed/@Pinterest_Engineering</t>
         </is>
       </c>
     </row>
@@ -2431,22 +2423,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>LWN.net</t>
+          <t>Shopify Engineering</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Linux kernel and open-source development</t>
+          <t>Commerce platform engineering at Shopify</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2455,14 +2447,14 @@
         </is>
       </c>
       <c r="G47" s="7" t="n">
-        <v>46321</v>
+        <v>46317</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>https://lwn.net/headlines/rss</t>
+          <t>https://shopify.engineering/blog.atom</t>
         </is>
       </c>
     </row>
@@ -2474,22 +2466,22 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Carbon Brief</t>
+          <t>Lyft Engineering</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Climate science and policy, data-driven</t>
+          <t>Marketplace, mapping and data engineering at Lyft</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -2498,14 +2490,14 @@
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>46318</v>
+        <v>46275</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>https://www.carbonbrief.org/feed/</t>
+          <t>https://eng.lyft.com/feed</t>
         </is>
       </c>
     </row>
@@ -2517,22 +2509,22 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Canary Media</t>
+          <t>Datadog Engineering</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Clean energy transition</t>
+          <t>Observability, distributed systems and security at Datadog</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -2541,14 +2533,14 @@
         </is>
       </c>
       <c r="G49" s="7" t="n">
-        <v>46322</v>
+        <v>46315</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>https://www.canarymedia.com/rss.rss</t>
+          <t>https://www.datadoghq.com/blog/engineering/index.xml</t>
         </is>
       </c>
     </row>
@@ -2560,22 +2552,22 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>CleanTechnica</t>
+          <t>GitHub Engineering</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Engineering blog</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>EVs, solar, clean tech (high volume)</t>
+          <t>How GitHub runs Git and its platform at scale</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -2584,14 +2576,14 @@
         </is>
       </c>
       <c r="G50" s="7" t="n">
-        <v>46322</v>
+        <v>46316</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>https://cleantechnica.com/feed/</t>
+          <t>https://github.blog/engineering/feed/</t>
         </is>
       </c>
     </row>
@@ -2603,22 +2595,22 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Electrek</t>
+          <t>ByteByteGo</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Newsletter</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>EVs and electric transport (high volume)</t>
+          <t>System design explainers on how big companies build their systems</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -2630,11 +2622,11 @@
         <v>46322</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>86</v>
+        <v>6</v>
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>https://electrek.co/feed/</t>
+          <t>https://blog.bytebytego.com/feed</t>
         </is>
       </c>
     </row>
@@ -2646,22 +2638,22 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Grist</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>International agency (via Google News)</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Climate and environmental justice</t>
+          <t>International Energy Agency reports, analysis and news</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -2673,11 +2665,11 @@
         <v>46322</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>https://grist.org/feed/</t>
+          <t>https://news.google.com/search?q=site%3Aiea.org%20when%3A30d</t>
         </is>
       </c>
     </row>
@@ -2689,12 +2681,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Inside Climate News</t>
+          <t>Carbon Brief</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -2704,7 +2696,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Investigative climate journalism</t>
+          <t>Climate science and policy, data-driven</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -2716,11 +2708,11 @@
         <v>46322</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>https://insideclimatenews.org/feed/</t>
+          <t>https://www.carbonbrief.org/feed/</t>
         </is>
       </c>
     </row>
@@ -2732,12 +2724,12 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>MIT Tech Review: Climate</t>
+          <t>Canary Media</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -2747,7 +2739,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Climate tech from MIT Technology Review</t>
+          <t>Clean energy transition</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -2759,11 +2751,11 @@
         <v>46322</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>https://www.technologyreview.com/topic/climate-change/feed</t>
+          <t>https://www.canarymedia.com/rss.rss</t>
         </is>
       </c>
     </row>
@@ -2775,12 +2767,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>DatacenterDynamics</t>
+          <t>CleanTechnica</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2790,7 +2782,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Data centres: power, cooling, energy use of AI</t>
+          <t>EVs, solar, clean tech (high volume)</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -2799,14 +2791,14 @@
         </is>
       </c>
       <c r="G55" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/rss/</t>
+          <t>https://cleantechnica.com/feed/</t>
         </is>
       </c>
     </row>
@@ -2818,22 +2810,22 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Krebs on Security</t>
+          <t>Electrek</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Expert blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Investigative cybercrime reporting</t>
+          <t>EVs and electric transport (high volume)</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -2842,14 +2834,14 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>https://krebsonsecurity.com/feed/</t>
+          <t>https://electrek.co/feed/</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2853,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>BleepingComputer</t>
+          <t>Grist</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2876,7 +2868,7 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Malware, breaches, vulnerabilities</t>
+          <t>Climate and environmental justice</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -2885,14 +2877,14 @@
         </is>
       </c>
       <c r="G57" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>https://www.bleepingcomputer.com/feed/</t>
+          <t>https://grist.org/feed/</t>
         </is>
       </c>
     </row>
@@ -2904,22 +2896,22 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Schneier on Security</t>
+          <t>Inside Climate News</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Expert blog</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Bruce Schneier on security and policy</t>
+          <t>Investigative climate journalism</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
@@ -2928,14 +2920,14 @@
         </is>
       </c>
       <c r="G58" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>https://www.schneier.com/feed/atom/</t>
+          <t>https://insideclimatenews.org/feed/</t>
         </is>
       </c>
     </row>
@@ -2947,12 +2939,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>The Hacker News</t>
+          <t>MIT Tech Review: Climate</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -2962,7 +2954,7 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Daily cybersecurity news</t>
+          <t>Climate tech from MIT Technology Review</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
@@ -2974,11 +2966,11 @@
         <v>46322</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>https://feeds.feedburner.com/TheHackersNews</t>
+          <t>https://www.technologyreview.com/topic/climate-change/feed</t>
         </is>
       </c>
     </row>
@@ -2990,12 +2982,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Hardware &amp; Chips</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Tom's Hardware</t>
+          <t>DatacenterDynamics</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -3005,7 +2997,7 @@
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>PC hardware, CPUs, GPUs (high volume)</t>
+          <t>Data centres: power, cooling, energy use of AI</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -3017,11 +3009,11 @@
         <v>46322</v>
       </c>
       <c r="H60" s="5" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/feeds/all</t>
+          <t>https://www.datacenterdynamics.com/en/rss/</t>
         </is>
       </c>
     </row>
@@ -3033,22 +3025,22 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Hardware &amp; Chips</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>IEEE Spectrum Semiconductors</t>
+          <t>Green Software Foundation</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Industry body</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Chip technology and fabrication</t>
+          <t>Standards and research on sustainable software</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -3057,14 +3049,14 @@
         </is>
       </c>
       <c r="G61" s="7" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="H61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>https://spectrum.ieee.org/feeds/topic/semiconductors.rss</t>
+          <t>https://greensoftware.foundation/rss.xml</t>
         </is>
       </c>
     </row>
@@ -3076,22 +3068,22 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Hardware &amp; Chips</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>ServeTheHome</t>
+          <t>Krebs on Security</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>News site</t>
+          <t>Expert blog</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>Servers, data-centre and AI hardware</t>
+          <t>Investigative cybercrime reporting</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -3100,14 +3092,14 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="H62" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>https://www.servethehome.com/feed/</t>
+          <t>https://krebsonsecurity.com/feed/</t>
         </is>
       </c>
     </row>
@@ -3119,22 +3111,22 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>MKBHD</t>
+          <t>BleepingComputer</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>Phone and gadget reviews</t>
+          <t>Malware, breaches, vulnerabilities</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -3143,14 +3135,14 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCBJycsmduvYEL83R_U4JriQ</t>
+          <t>https://www.bleepingcomputer.com/feed/</t>
         </is>
       </c>
     </row>
@@ -3162,22 +3154,22 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Linus Tech Tips</t>
+          <t>Schneier on Security</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>Expert blog</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>PC hardware, gadgets</t>
+          <t>Bruce Schneier on security and policy</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -3186,14 +3178,14 @@
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H64" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCXuqSBlHAE6Xw-yeJA0Tunw</t>
+          <t>https://www.schneier.com/feed/atom/</t>
         </is>
       </c>
     </row>
@@ -3205,22 +3197,22 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>The Verge</t>
+          <t>The Hacker News</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>Gadget reviews and tech explainers</t>
+          <t>Daily cybersecurity news</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
@@ -3229,14 +3221,14 @@
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H65" s="5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCddiUEpeqJcYeBxX1IVBKvQ</t>
+          <t>https://feeds.feedburner.com/TheHackersNews</t>
         </is>
       </c>
     </row>
@@ -3248,22 +3240,22 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Hardware &amp; Chips</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Dave2D</t>
+          <t>Tom's Hardware</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Laptop and gadget reviews</t>
+          <t>PC hardware, CPUs, GPUs (high volume)</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
@@ -3272,14 +3264,14 @@
         </is>
       </c>
       <c r="G66" s="7" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCVYamHliCI9rw1tHR1xbkfw</t>
+          <t>https://www.tomshardware.com/feeds/all</t>
         </is>
       </c>
     </row>
@@ -3291,22 +3283,22 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Hardware &amp; Chips</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Fireship</t>
+          <t>IEEE Spectrum Semiconductors</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Fast programming and dev-news videos</t>
+          <t>Chip technology and fabrication</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
@@ -3315,14 +3307,14 @@
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>46321</v>
+        <v>46318</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCsBjURrPoezykLs9EqgamOA</t>
+          <t>https://spectrum.ieee.org/feeds/topic/semiconductors.rss</t>
         </is>
       </c>
     </row>
@@ -3334,22 +3326,22 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Hardware &amp; Chips</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Two Minute Papers</t>
+          <t>ServeTheHome</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>AI and graphics research explained</t>
+          <t>Servers, data-centre and AI hardware</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
@@ -3358,14 +3350,14 @@
         </is>
       </c>
       <c r="G68" s="7" t="n">
-        <v>46314</v>
+        <v>46322</v>
       </c>
       <c r="H68" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCbfYPyITQ-7l4upoX8nvctg</t>
+          <t>https://www.servethehome.com/feed/</t>
         </is>
       </c>
     </row>
@@ -3377,22 +3369,22 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Yannic Kilcher</t>
+          <t>The Verge</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>ML paper walkthroughs</t>
+          <t>Consumer tech, gadgets, platforms, policy</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
@@ -3401,14 +3393,14 @@
         </is>
       </c>
       <c r="G69" s="7" t="n">
-        <v>46087</v>
+        <v>46322</v>
       </c>
       <c r="H69" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I69" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCZHmQk67mSJgfCCTn7xBfew</t>
+          <t>https://www.theverge.com/rss/index.xml</t>
         </is>
       </c>
     </row>
@@ -3420,22 +3412,22 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>AI Explained</t>
+          <t>TechCrunch</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Frontier AI model news and analysis</t>
+          <t>Startups, funding, venture capital, product launches</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
@@ -3444,14 +3436,14 @@
         </is>
       </c>
       <c r="G70" s="7" t="n">
-        <v>46307</v>
+        <v>46323</v>
       </c>
       <c r="H70" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCNJ1Ymd5yFuUPtn21xtRbbw</t>
+          <t>https://techcrunch.com/feed/</t>
         </is>
       </c>
     </row>
@@ -3463,22 +3455,22 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Andrej Karpathy</t>
+          <t>Ars Technica</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Deep LLM tutorials (posts rarely)</t>
+          <t>In-depth tech, science, IT and policy</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
@@ -3487,14 +3479,14 @@
         </is>
       </c>
       <c r="G71" s="7" t="n">
-        <v>45715</v>
+        <v>46322</v>
       </c>
       <c r="H71" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCXUPKJO5MZQN11PqgIvyuvQ</t>
+          <t>https://feeds.arstechnica.com/arstechnica/index</t>
         </is>
       </c>
     </row>
@@ -3506,22 +3498,22 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Machine Learning Street Talk</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Long-form AI research interviews</t>
+          <t>Tech culture, business, science, security</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -3530,14 +3522,14 @@
         </is>
       </c>
       <c r="G72" s="7" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="H72" s="5" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I72" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCMLtBahI5DMrt0NPvDSoIRQ</t>
+          <t>https://www.wired.com/feed/rss</t>
         </is>
       </c>
     </row>
@@ -3549,22 +3541,22 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Computerphile</t>
+          <t>Engadget</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Computer science concepts explained</t>
+          <t>Gadgets, gaming, consumer electronics</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
@@ -3573,14 +3565,14 @@
         </is>
       </c>
       <c r="G73" s="7" t="n">
-        <v>46317</v>
+        <v>46323</v>
       </c>
       <c r="H73" s="5" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="I73" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UC9-y-6csu5WGm29I7JiwpnA</t>
+          <t>https://www.engadget.com/rss.xml</t>
         </is>
       </c>
     </row>
@@ -3592,22 +3584,22 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>GOTO Conferences</t>
+          <t>The Register</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Software engineering conference talks</t>
+          <t>Enterprise IT, cloud, sysadmin, chips (UK)</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
@@ -3616,14 +3608,14 @@
         </is>
       </c>
       <c r="G74" s="7" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="H74" s="5" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCs_tLP3AiwYKwdUHpltJPuA</t>
+          <t>https://www.theregister.com/headlines.atom</t>
         </is>
       </c>
     </row>
@@ -3635,22 +3627,22 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Google for Developers</t>
+          <t>MIT Technology Review</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Google's official developer channel</t>
+          <t>Emerging tech, AI, biotech, climate tech</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
@@ -3659,14 +3651,14 @@
         </is>
       </c>
       <c r="G75" s="7" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="H75" s="5" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I75" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UC_x5XG1OV2P6uZZ5FSM9Ttw</t>
+          <t>https://www.technologyreview.com/feed/</t>
         </is>
       </c>
     </row>
@@ -3678,22 +3670,22 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Developer</t>
+          <t>Techmeme</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>Aggregator</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Microsoft's official developer channel</t>
+          <t>The day's top tech stories from across the web</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -3702,14 +3694,14 @@
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H76" s="5" t="n">
         <v>15</v>
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCsMica-v34Irf9KVTh6xx-g</t>
+          <t>https://www.techmeme.com/feed.xml</t>
         </is>
       </c>
     </row>
@@ -3721,22 +3713,22 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Hacker News (150+ pts)</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>Aggregator</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>NVIDIA's official channel</t>
+          <t>Popular Hacker News links (150+ points only)</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
@@ -3748,11 +3740,11 @@
         <v>46322</v>
       </c>
       <c r="H77" s="5" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I77" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCHuiy8bXnmK5nisYHUd1J5g</t>
+          <t>https://hnrss.org/frontpage?points=150</t>
         </is>
       </c>
     </row>
@@ -3764,22 +3756,22 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Rest of World</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Apple's official channel (events, ads)</t>
+          <t>Tech outside the US and Europe (Asia, Africa, LatAm)</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -3795,7 +3787,7 @@
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCE_M8A5yxnLfW0KghEeajjw</t>
+          <t>https://restofworld.org/feed/latest</t>
         </is>
       </c>
     </row>
@@ -3807,22 +3799,22 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Lex Fridman</t>
+          <t>The Next Web</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Long interviews with tech and AI people</t>
+          <t>European tech, startups, deep tech</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
@@ -3831,14 +3823,14 @@
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H79" s="5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I79" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCSHZKyawb77ixDdsGog4iWA</t>
+          <t>https://thenextweb.com/feed</t>
         </is>
       </c>
     </row>
@@ -3850,22 +3842,22 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Tech News</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Undecided with Matt Ferrell</t>
+          <t>9to5Mac</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>YouTube channel</t>
+          <t>News site</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Clean energy and sustainable tech</t>
+          <t>Apple, iPhone, Mac (high volume)</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
@@ -3874,14 +3866,14 @@
         </is>
       </c>
       <c r="G80" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H80" s="5" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I80" s="8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCjtUS7-SZTi6pXjUbzGHQCg</t>
+          <t>https://9to5mac.com/feed/</t>
         </is>
       </c>
     </row>
@@ -3893,172 +3885,913 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
+          <t>Tech News</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>9to5Google</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>News site</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Google, Android, Pixel (high volume)</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H81" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>https://9to5google.com/feed/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
           <t>Videos</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>MKBHD</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Phone and gadget reviews</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="n"/>
+      <c r="H82" s="5" t="n"/>
+      <c r="I82" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCBJycsmduvYEL83R_U4JriQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Linus Tech Tips</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>PC hardware, gadgets</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="n"/>
+      <c r="H83" s="5" t="n"/>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCXuqSBlHAE6Xw-yeJA0Tunw</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>The Verge</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>Gadget reviews and tech explainers</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="n"/>
+      <c r="H84" s="5" t="n"/>
+      <c r="I84" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCddiUEpeqJcYeBxX1IVBKvQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Dave2D</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>Laptop and gadget reviews</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="n"/>
+      <c r="H85" s="5" t="n"/>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCVYamHliCI9rw1tHR1xbkfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Fireship</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>Fast programming and dev-news videos</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="n"/>
+      <c r="H86" s="5" t="n"/>
+      <c r="I86" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCsBjURrPoezykLs9EqgamOA</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Two Minute Papers</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>AI and graphics research explained</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="n"/>
+      <c r="H87" s="5" t="n"/>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCbfYPyITQ-7l4upoX8nvctg</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Yannic Kilcher</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>ML paper walkthroughs</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="n"/>
+      <c r="H88" s="5" t="n"/>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCZHmQk67mSJgfCCTn7xBfew</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>AI Explained</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>Frontier AI model news and analysis</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="n"/>
+      <c r="H89" s="5" t="n"/>
+      <c r="I89" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCNJ1Ymd5yFuUPtn21xtRbbw</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Andrej Karpathy</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E90" s="6" t="inlineStr">
+        <is>
+          <t>Deep LLM tutorials (posts rarely)</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="n"/>
+      <c r="H90" s="5" t="n"/>
+      <c r="I90" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCXUPKJO5MZQN11PqgIvyuvQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Machine Learning Street Talk</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Long-form AI research interviews</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="n"/>
+      <c r="H91" s="5" t="n"/>
+      <c r="I91" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCMLtBahI5DMrt0NPvDSoIRQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Computerphile</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="inlineStr">
+        <is>
+          <t>Computer science concepts explained</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="n"/>
+      <c r="H92" s="5" t="n"/>
+      <c r="I92" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UC9-y-6csu5WGm29I7JiwpnA</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>GOTO Conferences</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>Software engineering conference talks</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="n"/>
+      <c r="H93" s="5" t="n"/>
+      <c r="I93" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCs_tLP3AiwYKwdUHpltJPuA</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Google for Developers</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr">
+        <is>
+          <t>Google's official developer channel</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="n"/>
+      <c r="H94" s="5" t="n"/>
+      <c r="I94" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UC_x5XG1OV2P6uZZ5FSM9Ttw</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft Developer</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft's official developer channel</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="n"/>
+      <c r="H95" s="5" t="n"/>
+      <c r="I95" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCsMica-v34Irf9KVTh6xx-g</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>NVIDIA's official channel</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="n"/>
+      <c r="H96" s="5" t="n"/>
+      <c r="I96" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCHuiy8bXnmK5nisYHUd1J5g</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>Apple's official channel (events, ads)</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="n"/>
+      <c r="H97" s="5" t="n"/>
+      <c r="I97" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCE_M8A5yxnLfW0KghEeajjw</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Lex Fridman</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>Long interviews with tech and AI people</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="n"/>
+      <c r="H98" s="5" t="n"/>
+      <c r="I98" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCSHZKyawb77ixDdsGog4iWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Undecided with Matt Ferrell</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Clean energy and sustainable tech</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="n"/>
+      <c r="H99" s="5" t="n"/>
+      <c r="I99" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCjtUS7-SZTi6pXjUbzGHQCg</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>Climate Town</t>
         </is>
       </c>
-      <c r="D81" s="5" t="inlineStr">
+      <c r="D100" s="5" t="inlineStr">
         <is>
           <t>YouTube channel</t>
         </is>
       </c>
-      <c r="E81" s="6" t="inlineStr">
+      <c r="E100" s="6" t="inlineStr">
         <is>
           <t>Climate explained with humour</t>
         </is>
       </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G81" s="7" t="n">
-        <v>46303</v>
-      </c>
-      <c r="H81" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" s="8" t="inlineStr">
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Not checked: YouTube feeds were down during this check</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="n"/>
+      <c r="H100" s="5" t="n"/>
+      <c r="I100" s="8" t="inlineStr">
         <is>
           <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCuVLG9pThvBABcYCm7pkNkA</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="9" t="n"/>
-      <c r="B82" s="10" t="n"/>
-      <c r="C82" s="11" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="9" t="n"/>
+      <c r="B101" s="10" t="n"/>
+      <c r="C101" s="11" t="inlineStr">
         <is>
           <t>(add your own here)</t>
         </is>
       </c>
-      <c r="D82" s="10" t="n"/>
-      <c r="E82" s="10" t="n"/>
-      <c r="F82" s="10" t="n"/>
-      <c r="G82" s="10" t="n"/>
-      <c r="H82" s="10" t="n"/>
-      <c r="I82" s="10" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="9" t="n"/>
-      <c r="B83" s="10" t="n"/>
-      <c r="C83" s="10" t="n"/>
-      <c r="D83" s="10" t="n"/>
-      <c r="E83" s="10" t="n"/>
-      <c r="F83" s="10" t="n"/>
-      <c r="G83" s="10" t="n"/>
-      <c r="H83" s="10" t="n"/>
-      <c r="I83" s="10" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="9" t="n"/>
-      <c r="B84" s="10" t="n"/>
-      <c r="C84" s="10" t="n"/>
-      <c r="D84" s="10" t="n"/>
-      <c r="E84" s="10" t="n"/>
-      <c r="F84" s="10" t="n"/>
-      <c r="G84" s="10" t="n"/>
-      <c r="H84" s="10" t="n"/>
-      <c r="I84" s="10" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="9" t="n"/>
-      <c r="B85" s="10" t="n"/>
-      <c r="C85" s="10" t="n"/>
-      <c r="D85" s="10" t="n"/>
-      <c r="E85" s="10" t="n"/>
-      <c r="F85" s="10" t="n"/>
-      <c r="G85" s="10" t="n"/>
-      <c r="H85" s="10" t="n"/>
-      <c r="I85" s="10" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="9" t="n"/>
-      <c r="B86" s="10" t="n"/>
-      <c r="C86" s="10" t="n"/>
-      <c r="D86" s="10" t="n"/>
-      <c r="E86" s="10" t="n"/>
-      <c r="F86" s="10" t="n"/>
-      <c r="G86" s="10" t="n"/>
-      <c r="H86" s="10" t="n"/>
-      <c r="I86" s="10" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="9" t="n"/>
-      <c r="B87" s="10" t="n"/>
-      <c r="C87" s="10" t="n"/>
-      <c r="D87" s="10" t="n"/>
-      <c r="E87" s="10" t="n"/>
-      <c r="F87" s="10" t="n"/>
-      <c r="G87" s="10" t="n"/>
-      <c r="H87" s="10" t="n"/>
-      <c r="I87" s="10" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="9" t="n"/>
-      <c r="B88" s="10" t="n"/>
-      <c r="C88" s="10" t="n"/>
-      <c r="D88" s="10" t="n"/>
-      <c r="E88" s="10" t="n"/>
-      <c r="F88" s="10" t="n"/>
-      <c r="G88" s="10" t="n"/>
-      <c r="H88" s="10" t="n"/>
-      <c r="I88" s="10" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="9" t="n"/>
-      <c r="B89" s="10" t="n"/>
-      <c r="C89" s="10" t="n"/>
-      <c r="D89" s="10" t="n"/>
-      <c r="E89" s="10" t="n"/>
-      <c r="F89" s="10" t="n"/>
-      <c r="G89" s="10" t="n"/>
-      <c r="H89" s="10" t="n"/>
-      <c r="I89" s="10" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="9" t="n"/>
-      <c r="B90" s="10" t="n"/>
-      <c r="C90" s="10" t="n"/>
-      <c r="D90" s="10" t="n"/>
-      <c r="E90" s="10" t="n"/>
-      <c r="F90" s="10" t="n"/>
-      <c r="G90" s="10" t="n"/>
-      <c r="H90" s="10" t="n"/>
-      <c r="I90" s="10" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="9" t="n"/>
-      <c r="B91" s="10" t="n"/>
-      <c r="C91" s="10" t="n"/>
-      <c r="D91" s="10" t="n"/>
-      <c r="E91" s="10" t="n"/>
-      <c r="F91" s="10" t="n"/>
-      <c r="G91" s="10" t="n"/>
-      <c r="H91" s="10" t="n"/>
-      <c r="I91" s="10" t="n"/>
+      <c r="D101" s="10" t="n"/>
+      <c r="E101" s="10" t="n"/>
+      <c r="F101" s="10" t="n"/>
+      <c r="G101" s="10" t="n"/>
+      <c r="H101" s="10" t="n"/>
+      <c r="I101" s="10" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="9" t="n"/>
+      <c r="B102" s="10" t="n"/>
+      <c r="C102" s="10" t="n"/>
+      <c r="D102" s="10" t="n"/>
+      <c r="E102" s="10" t="n"/>
+      <c r="F102" s="10" t="n"/>
+      <c r="G102" s="10" t="n"/>
+      <c r="H102" s="10" t="n"/>
+      <c r="I102" s="10" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="n"/>
+      <c r="B103" s="10" t="n"/>
+      <c r="C103" s="10" t="n"/>
+      <c r="D103" s="10" t="n"/>
+      <c r="E103" s="10" t="n"/>
+      <c r="F103" s="10" t="n"/>
+      <c r="G103" s="10" t="n"/>
+      <c r="H103" s="10" t="n"/>
+      <c r="I103" s="10" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="9" t="n"/>
+      <c r="B104" s="10" t="n"/>
+      <c r="C104" s="10" t="n"/>
+      <c r="D104" s="10" t="n"/>
+      <c r="E104" s="10" t="n"/>
+      <c r="F104" s="10" t="n"/>
+      <c r="G104" s="10" t="n"/>
+      <c r="H104" s="10" t="n"/>
+      <c r="I104" s="10" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="9" t="n"/>
+      <c r="B105" s="10" t="n"/>
+      <c r="C105" s="10" t="n"/>
+      <c r="D105" s="10" t="n"/>
+      <c r="E105" s="10" t="n"/>
+      <c r="F105" s="10" t="n"/>
+      <c r="G105" s="10" t="n"/>
+      <c r="H105" s="10" t="n"/>
+      <c r="I105" s="10" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="n"/>
+      <c r="B106" s="10" t="n"/>
+      <c r="C106" s="10" t="n"/>
+      <c r="D106" s="10" t="n"/>
+      <c r="E106" s="10" t="n"/>
+      <c r="F106" s="10" t="n"/>
+      <c r="G106" s="10" t="n"/>
+      <c r="H106" s="10" t="n"/>
+      <c r="I106" s="10" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="9" t="n"/>
+      <c r="B107" s="10" t="n"/>
+      <c r="C107" s="10" t="n"/>
+      <c r="D107" s="10" t="n"/>
+      <c r="E107" s="10" t="n"/>
+      <c r="F107" s="10" t="n"/>
+      <c r="G107" s="10" t="n"/>
+      <c r="H107" s="10" t="n"/>
+      <c r="I107" s="10" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="9" t="n"/>
+      <c r="B108" s="10" t="n"/>
+      <c r="C108" s="10" t="n"/>
+      <c r="D108" s="10" t="n"/>
+      <c r="E108" s="10" t="n"/>
+      <c r="F108" s="10" t="n"/>
+      <c r="G108" s="10" t="n"/>
+      <c r="H108" s="10" t="n"/>
+      <c r="I108" s="10" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="n"/>
+      <c r="B109" s="10" t="n"/>
+      <c r="C109" s="10" t="n"/>
+      <c r="D109" s="10" t="n"/>
+      <c r="E109" s="10" t="n"/>
+      <c r="F109" s="10" t="n"/>
+      <c r="G109" s="10" t="n"/>
+      <c r="H109" s="10" t="n"/>
+      <c r="I109" s="10" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="n"/>
+      <c r="B110" s="10" t="n"/>
+      <c r="C110" s="10" t="n"/>
+      <c r="D110" s="10" t="n"/>
+      <c r="E110" s="10" t="n"/>
+      <c r="F110" s="10" t="n"/>
+      <c r="G110" s="10" t="n"/>
+      <c r="H110" s="10" t="n"/>
+      <c r="I110" s="10" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I91"/>
+  <autoFilter ref="A4:I110"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:I91">
+  <conditionalFormatting sqref="A5:I110">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$A5="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F91">
+  <conditionalFormatting sqref="F5:F110">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>LEFT($F5,2)="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5:A91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A5:A110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4095,7 +4828,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Conferences: papers whose authors note on arXiv that they were accepted there (this year and next). Journals: newest 60 articles with abstracts (OpenAlex). Topics: newest arXiv papers matching a search. Counts are from 27 Oct 2026. Set Include? to Yes or No; add venues in the blank rows.</t>
+          <t>Conferences: papers whose authors note on arXiv that they were accepted there (this year and next). Journals: newest 60 articles with abstracts (OpenAlex). Topics: newest arXiv papers matching a search. Counts are from 28 Oct 2026. Set Include? to Yes or No; add venues in the blank rows.</t>
         </is>
       </c>
     </row>
@@ -5589,7 +6322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5634,30 +6367,30 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Tech News</t>
+          <t>Big Tech &amp; Labs</t>
         </is>
       </c>
       <c r="B5" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A5)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A5)</f>
         <v/>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A5,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A5,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>Big Tech</t>
+          <t>Model Watch</t>
         </is>
       </c>
       <c r="B6" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A6)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A6)</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A6,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A6,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -5668,11 +6401,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A7)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A7)</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A7,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A7,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -5683,131 +6416,161 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A8)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A8)</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A8,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A8,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Engineering Blogs</t>
         </is>
       </c>
       <c r="B9" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A9)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A9)</f>
         <v/>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A9,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A9,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Sustainability &amp; Energy</t>
         </is>
       </c>
       <c r="B10" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A10)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A10)</f>
         <v/>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A10,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A10,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Hardware &amp; Chips</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B11" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A11)</f>
+        <f>COUNTIF(Sources!$B$5:$B$110,A11)</f>
         <v/>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A11,Sources!$A$5:$A$91,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$110,A11,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
+          <t>Hardware &amp; Chips</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>COUNTIF(Sources!$B$5:$B$110,A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="15">
+        <f>COUNTIFS(Sources!$B$5:$B$110,A12,Sources!$A$5:$A$110,"Yes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Tech News</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>COUNTIF(Sources!$B$5:$B$110,A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="15">
+        <f>COUNTIFS(Sources!$B$5:$B$110,A13,Sources!$A$5:$A$110,"Yes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
           <t>Videos</t>
         </is>
       </c>
-      <c r="B12" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$91,A12)</f>
+      <c r="B14" s="15">
+        <f>COUNTIF(Sources!$B$5:$B$110,A14)</f>
         <v/>
       </c>
-      <c r="C12" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$91,A12,Sources!$A$5:$A$91,"Yes")</f>
+      <c r="C14" s="15">
+        <f>COUNTIFS(Sources!$B$5:$B$110,A14,Sources!$A$5:$A$110,"Yes")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B13" s="16">
-        <f>SUM(B5:B12)</f>
+      <c r="B15" s="16">
+        <f>SUM(B5:B14)</f>
         <v/>
       </c>
-      <c r="C13" s="16">
-        <f>SUM(C5:C12)</f>
+      <c r="C15" s="16">
+        <f>SUM(C5:C14)</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Anthropic, Meta AI (ai.meta.com) and The Batch (DeepLearning.AI) publish no RSS feed, so they can't be followed automatically. Their stories still show up through Techmeme, The Verge, The Decoder and others.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>arXiv searches are tuned to your research (agents, AI for SE, LLM energy, uncertainty). Tell me other keywords and I'll add them.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>Any YouTube channel can be added: give me the channel link.</t>
+          <t>Anthropic, Meta AI (ai.meta.com) and The Batch (DeepLearning.AI) publish no RSS feed, so they can't be followed automatically. Their stories still show up through Techmeme, The Verge, The Decoder and others.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="18" t="inlineStr">
         <is>
+          <t>arXiv searches are tuned to your research (agents, AI for SE, LLM energy, uncertainty). Tell me other keywords and I'll add them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Any YouTube channel can be added: give me the channel link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
           <t>The site updates itself every hour: new posts from every chosen source appear on their own.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Videos; IEA shows only its reports, linked straight to iea.org; Research tab and sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tech-Pulse-Sources.xlsx
+++ b/Tech-Pulse-Sources.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Paper venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Research papers" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$4:$I$110</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Paper venues'!$A$4:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$4:$I$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Research papers'!$A$4:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -559,14 +559,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tech Pulse: candidate sources</t>
+          <t>Tech Pulse: news sources (research papers are on the next sheet, "Research papers")</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How to use: in the yellow 'Include?' column, choose Yes or No for each source. Add your own sources at the bottom (any site with an RSS feed, or any YouTube channel). Every feed was tested on 28 Oct 2026.</t>
+          <t>How to use: in the yellow 'Include?' column, choose Yes or No for each source. Add your own sources at the bottom (any site with an RSS feed). Conferences, journals and arXiv topic searches are on the "Research papers" sheet. Every feed was tested on 28 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
         <v>46322</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -993,10 +993,10 @@
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H20" s="5" t="n">
         <v>12</v>
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="G28" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H28" s="5" t="n">
         <v>10</v>
@@ -2665,11 +2665,11 @@
         <v>46322</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>https://news.google.com/search?q=site%3Aiea.org%20when%3A30d</t>
+          <t>https://news.google.com/search?q=site%3Aiea.org/reports%20when%3A30d</t>
         </is>
       </c>
     </row>
@@ -2705,10 +2705,10 @@
         </is>
       </c>
       <c r="G53" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
@@ -2748,10 +2748,10 @@
         </is>
       </c>
       <c r="G54" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
@@ -2834,7 +2834,7 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H56" s="5" t="n">
         <v>25</v>
@@ -2880,7 +2880,7 @@
         <v>46323</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H65" s="5" t="n">
         <v>25</v>
@@ -3737,10 +3737,10 @@
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H77" s="5" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I77" s="8" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H79" s="5" t="n">
         <v>10</v>
@@ -3921,877 +3921,136 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>MKBHD</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E82" s="6" t="inlineStr">
-        <is>
-          <t>Phone and gadget reviews</t>
-        </is>
-      </c>
-      <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G82" s="7" t="n"/>
-      <c r="H82" s="5" t="n"/>
-      <c r="I82" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCBJycsmduvYEL83R_U4JriQ</t>
-        </is>
-      </c>
+      <c r="A82" s="9" t="n"/>
+      <c r="B82" s="10" t="n"/>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>(add your own here)</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="n"/>
+      <c r="E82" s="10" t="n"/>
+      <c r="F82" s="10" t="n"/>
+      <c r="G82" s="10" t="n"/>
+      <c r="H82" s="10" t="n"/>
+      <c r="I82" s="10" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>Linus Tech Tips</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E83" s="6" t="inlineStr">
-        <is>
-          <t>PC hardware, gadgets</t>
-        </is>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G83" s="7" t="n"/>
-      <c r="H83" s="5" t="n"/>
-      <c r="I83" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCXuqSBlHAE6Xw-yeJA0Tunw</t>
-        </is>
-      </c>
+      <c r="A83" s="9" t="n"/>
+      <c r="B83" s="10" t="n"/>
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="10" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="10" t="n"/>
+      <c r="G83" s="10" t="n"/>
+      <c r="H83" s="10" t="n"/>
+      <c r="I83" s="10" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>The Verge</t>
-        </is>
-      </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E84" s="6" t="inlineStr">
-        <is>
-          <t>Gadget reviews and tech explainers</t>
-        </is>
-      </c>
-      <c r="F84" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G84" s="7" t="n"/>
-      <c r="H84" s="5" t="n"/>
-      <c r="I84" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCddiUEpeqJcYeBxX1IVBKvQ</t>
-        </is>
-      </c>
+      <c r="A84" s="9" t="n"/>
+      <c r="B84" s="10" t="n"/>
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="10" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+      <c r="G84" s="10" t="n"/>
+      <c r="H84" s="10" t="n"/>
+      <c r="I84" s="10" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>Dave2D</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E85" s="6" t="inlineStr">
-        <is>
-          <t>Laptop and gadget reviews</t>
-        </is>
-      </c>
-      <c r="F85" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="n"/>
-      <c r="H85" s="5" t="n"/>
-      <c r="I85" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCVYamHliCI9rw1tHR1xbkfw</t>
-        </is>
-      </c>
+      <c r="A85" s="9" t="n"/>
+      <c r="B85" s="10" t="n"/>
+      <c r="C85" s="10" t="n"/>
+      <c r="D85" s="10" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="10" t="n"/>
+      <c r="G85" s="10" t="n"/>
+      <c r="H85" s="10" t="n"/>
+      <c r="I85" s="10" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>Fireship</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E86" s="6" t="inlineStr">
-        <is>
-          <t>Fast programming and dev-news videos</t>
-        </is>
-      </c>
-      <c r="F86" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="n"/>
-      <c r="H86" s="5" t="n"/>
-      <c r="I86" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCsBjURrPoezykLs9EqgamOA</t>
-        </is>
-      </c>
+      <c r="A86" s="9" t="n"/>
+      <c r="B86" s="10" t="n"/>
+      <c r="C86" s="10" t="n"/>
+      <c r="D86" s="10" t="n"/>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="10" t="n"/>
+      <c r="G86" s="10" t="n"/>
+      <c r="H86" s="10" t="n"/>
+      <c r="I86" s="10" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>Two Minute Papers</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E87" s="6" t="inlineStr">
-        <is>
-          <t>AI and graphics research explained</t>
-        </is>
-      </c>
-      <c r="F87" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G87" s="7" t="n"/>
-      <c r="H87" s="5" t="n"/>
-      <c r="I87" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCbfYPyITQ-7l4upoX8nvctg</t>
-        </is>
-      </c>
+      <c r="A87" s="9" t="n"/>
+      <c r="B87" s="10" t="n"/>
+      <c r="C87" s="10" t="n"/>
+      <c r="D87" s="10" t="n"/>
+      <c r="E87" s="10" t="n"/>
+      <c r="F87" s="10" t="n"/>
+      <c r="G87" s="10" t="n"/>
+      <c r="H87" s="10" t="n"/>
+      <c r="I87" s="10" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>Yannic Kilcher</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E88" s="6" t="inlineStr">
-        <is>
-          <t>ML paper walkthroughs</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G88" s="7" t="n"/>
-      <c r="H88" s="5" t="n"/>
-      <c r="I88" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCZHmQk67mSJgfCCTn7xBfew</t>
-        </is>
-      </c>
+      <c r="A88" s="9" t="n"/>
+      <c r="B88" s="10" t="n"/>
+      <c r="C88" s="10" t="n"/>
+      <c r="D88" s="10" t="n"/>
+      <c r="E88" s="10" t="n"/>
+      <c r="F88" s="10" t="n"/>
+      <c r="G88" s="10" t="n"/>
+      <c r="H88" s="10" t="n"/>
+      <c r="I88" s="10" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>AI Explained</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E89" s="6" t="inlineStr">
-        <is>
-          <t>Frontier AI model news and analysis</t>
-        </is>
-      </c>
-      <c r="F89" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G89" s="7" t="n"/>
-      <c r="H89" s="5" t="n"/>
-      <c r="I89" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCNJ1Ymd5yFuUPtn21xtRbbw</t>
-        </is>
-      </c>
+      <c r="A89" s="9" t="n"/>
+      <c r="B89" s="10" t="n"/>
+      <c r="C89" s="10" t="n"/>
+      <c r="D89" s="10" t="n"/>
+      <c r="E89" s="10" t="n"/>
+      <c r="F89" s="10" t="n"/>
+      <c r="G89" s="10" t="n"/>
+      <c r="H89" s="10" t="n"/>
+      <c r="I89" s="10" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>Andrej Karpathy</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E90" s="6" t="inlineStr">
-        <is>
-          <t>Deep LLM tutorials (posts rarely)</t>
-        </is>
-      </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G90" s="7" t="n"/>
-      <c r="H90" s="5" t="n"/>
-      <c r="I90" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCXUPKJO5MZQN11PqgIvyuvQ</t>
-        </is>
-      </c>
+      <c r="A90" s="9" t="n"/>
+      <c r="B90" s="10" t="n"/>
+      <c r="C90" s="10" t="n"/>
+      <c r="D90" s="10" t="n"/>
+      <c r="E90" s="10" t="n"/>
+      <c r="F90" s="10" t="n"/>
+      <c r="G90" s="10" t="n"/>
+      <c r="H90" s="10" t="n"/>
+      <c r="I90" s="10" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>Machine Learning Street Talk</t>
-        </is>
-      </c>
-      <c r="D91" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E91" s="6" t="inlineStr">
-        <is>
-          <t>Long-form AI research interviews</t>
-        </is>
-      </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="n"/>
-      <c r="H91" s="5" t="n"/>
-      <c r="I91" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCMLtBahI5DMrt0NPvDSoIRQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B92" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>Computerphile</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E92" s="6" t="inlineStr">
-        <is>
-          <t>Computer science concepts explained</t>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="n"/>
-      <c r="H92" s="5" t="n"/>
-      <c r="I92" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UC9-y-6csu5WGm29I7JiwpnA</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B93" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>GOTO Conferences</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
-        <is>
-          <t>Software engineering conference talks</t>
-        </is>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="n"/>
-      <c r="H93" s="5" t="n"/>
-      <c r="I93" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCs_tLP3AiwYKwdUHpltJPuA</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>Google for Developers</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E94" s="6" t="inlineStr">
-        <is>
-          <t>Google's official developer channel</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="n"/>
-      <c r="H94" s="5" t="n"/>
-      <c r="I94" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UC_x5XG1OV2P6uZZ5FSM9Ttw</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>Microsoft Developer</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E95" s="6" t="inlineStr">
-        <is>
-          <t>Microsoft's official developer channel</t>
-        </is>
-      </c>
-      <c r="F95" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="n"/>
-      <c r="H95" s="5" t="n"/>
-      <c r="I95" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCsMica-v34Irf9KVTh6xx-g</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>NVIDIA</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
-        <is>
-          <t>NVIDIA's official channel</t>
-        </is>
-      </c>
-      <c r="F96" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G96" s="7" t="n"/>
-      <c r="H96" s="5" t="n"/>
-      <c r="I96" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCHuiy8bXnmK5nisYHUd1J5g</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>Apple</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="inlineStr">
-        <is>
-          <t>Apple's official channel (events, ads)</t>
-        </is>
-      </c>
-      <c r="F97" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G97" s="7" t="n"/>
-      <c r="H97" s="5" t="n"/>
-      <c r="I97" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCE_M8A5yxnLfW0KghEeajjw</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>Lex Fridman</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="inlineStr">
-        <is>
-          <t>Long interviews with tech and AI people</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G98" s="7" t="n"/>
-      <c r="H98" s="5" t="n"/>
-      <c r="I98" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCSHZKyawb77ixDdsGog4iWA</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>Undecided with Matt Ferrell</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E99" s="6" t="inlineStr">
-        <is>
-          <t>Clean energy and sustainable tech</t>
-        </is>
-      </c>
-      <c r="F99" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G99" s="7" t="n"/>
-      <c r="H99" s="5" t="n"/>
-      <c r="I99" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCjtUS7-SZTi6pXjUbzGHQCg</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B100" s="5" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>Climate Town</t>
-        </is>
-      </c>
-      <c r="D100" s="5" t="inlineStr">
-        <is>
-          <t>YouTube channel</t>
-        </is>
-      </c>
-      <c r="E100" s="6" t="inlineStr">
-        <is>
-          <t>Climate explained with humour</t>
-        </is>
-      </c>
-      <c r="F100" s="5" t="inlineStr">
-        <is>
-          <t>Not checked: YouTube feeds were down during this check</t>
-        </is>
-      </c>
-      <c r="G100" s="7" t="n"/>
-      <c r="H100" s="5" t="n"/>
-      <c r="I100" s="8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/feeds/videos.xml?channel_id=UCuVLG9pThvBABcYCm7pkNkA</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="9" t="n"/>
-      <c r="B101" s="10" t="n"/>
-      <c r="C101" s="11" t="inlineStr">
-        <is>
-          <t>(add your own here)</t>
-        </is>
-      </c>
-      <c r="D101" s="10" t="n"/>
-      <c r="E101" s="10" t="n"/>
-      <c r="F101" s="10" t="n"/>
-      <c r="G101" s="10" t="n"/>
-      <c r="H101" s="10" t="n"/>
-      <c r="I101" s="10" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="9" t="n"/>
-      <c r="B102" s="10" t="n"/>
-      <c r="C102" s="10" t="n"/>
-      <c r="D102" s="10" t="n"/>
-      <c r="E102" s="10" t="n"/>
-      <c r="F102" s="10" t="n"/>
-      <c r="G102" s="10" t="n"/>
-      <c r="H102" s="10" t="n"/>
-      <c r="I102" s="10" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="9" t="n"/>
-      <c r="B103" s="10" t="n"/>
-      <c r="C103" s="10" t="n"/>
-      <c r="D103" s="10" t="n"/>
-      <c r="E103" s="10" t="n"/>
-      <c r="F103" s="10" t="n"/>
-      <c r="G103" s="10" t="n"/>
-      <c r="H103" s="10" t="n"/>
-      <c r="I103" s="10" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="9" t="n"/>
-      <c r="B104" s="10" t="n"/>
-      <c r="C104" s="10" t="n"/>
-      <c r="D104" s="10" t="n"/>
-      <c r="E104" s="10" t="n"/>
-      <c r="F104" s="10" t="n"/>
-      <c r="G104" s="10" t="n"/>
-      <c r="H104" s="10" t="n"/>
-      <c r="I104" s="10" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="9" t="n"/>
-      <c r="B105" s="10" t="n"/>
-      <c r="C105" s="10" t="n"/>
-      <c r="D105" s="10" t="n"/>
-      <c r="E105" s="10" t="n"/>
-      <c r="F105" s="10" t="n"/>
-      <c r="G105" s="10" t="n"/>
-      <c r="H105" s="10" t="n"/>
-      <c r="I105" s="10" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="9" t="n"/>
-      <c r="B106" s="10" t="n"/>
-      <c r="C106" s="10" t="n"/>
-      <c r="D106" s="10" t="n"/>
-      <c r="E106" s="10" t="n"/>
-      <c r="F106" s="10" t="n"/>
-      <c r="G106" s="10" t="n"/>
-      <c r="H106" s="10" t="n"/>
-      <c r="I106" s="10" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="9" t="n"/>
-      <c r="B107" s="10" t="n"/>
-      <c r="C107" s="10" t="n"/>
-      <c r="D107" s="10" t="n"/>
-      <c r="E107" s="10" t="n"/>
-      <c r="F107" s="10" t="n"/>
-      <c r="G107" s="10" t="n"/>
-      <c r="H107" s="10" t="n"/>
-      <c r="I107" s="10" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="9" t="n"/>
-      <c r="B108" s="10" t="n"/>
-      <c r="C108" s="10" t="n"/>
-      <c r="D108" s="10" t="n"/>
-      <c r="E108" s="10" t="n"/>
-      <c r="F108" s="10" t="n"/>
-      <c r="G108" s="10" t="n"/>
-      <c r="H108" s="10" t="n"/>
-      <c r="I108" s="10" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="9" t="n"/>
-      <c r="B109" s="10" t="n"/>
-      <c r="C109" s="10" t="n"/>
-      <c r="D109" s="10" t="n"/>
-      <c r="E109" s="10" t="n"/>
-      <c r="F109" s="10" t="n"/>
-      <c r="G109" s="10" t="n"/>
-      <c r="H109" s="10" t="n"/>
-      <c r="I109" s="10" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="9" t="n"/>
-      <c r="B110" s="10" t="n"/>
-      <c r="C110" s="10" t="n"/>
-      <c r="D110" s="10" t="n"/>
-      <c r="E110" s="10" t="n"/>
-      <c r="F110" s="10" t="n"/>
-      <c r="G110" s="10" t="n"/>
-      <c r="H110" s="10" t="n"/>
-      <c r="I110" s="10" t="n"/>
+      <c r="A91" s="9" t="n"/>
+      <c r="B91" s="10" t="n"/>
+      <c r="C91" s="10" t="n"/>
+      <c r="D91" s="10" t="n"/>
+      <c r="E91" s="10" t="n"/>
+      <c r="F91" s="10" t="n"/>
+      <c r="G91" s="10" t="n"/>
+      <c r="H91" s="10" t="n"/>
+      <c r="I91" s="10" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I110"/>
+  <autoFilter ref="A4:I91"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:I110">
+  <conditionalFormatting sqref="A5:I91">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$A5="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F110">
+  <conditionalFormatting sqref="F5:F91">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>LEFT($F5,2)="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5:A110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A5:A91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6322,7 +5581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6371,11 +5630,11 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A5)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A5)</f>
         <v/>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A5,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A5,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6386,11 +5645,11 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A6)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A6)</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A6,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A6,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6401,11 +5660,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A7)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A7)</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A7,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A7,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6416,11 +5675,11 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A8)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A8)</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A8,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A8,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6431,11 +5690,11 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A9)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A9)</f>
         <v/>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A9,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A9,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6446,11 +5705,11 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A10)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A10)</f>
         <v/>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A10,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A10,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6461,11 +5720,11 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A11)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A11)</f>
         <v/>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A11,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A11,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6476,11 +5735,11 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A12)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A12)</f>
         <v/>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A12,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A12,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -6491,74 +5750,104 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A13)</f>
+        <f>COUNTIF(Sources!$B$5:$B$91,A13)</f>
         <v/>
       </c>
       <c r="C13" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A13,Sources!$A$5:$A$110,"Yes")</f>
+        <f>COUNTIFS(Sources!$B$5:$B$91,A13,Sources!$A$5:$A$91,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Videos</t>
-        </is>
-      </c>
-      <c r="B14" s="15">
-        <f>COUNTIF(Sources!$B$5:$B$110,A14)</f>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B14" s="16">
+        <f>SUM(B5:B13)</f>
         <v/>
       </c>
-      <c r="C14" s="15">
-        <f>COUNTIFS(Sources!$B$5:$B$110,A14,Sources!$A$5:$A$110,"Yes")</f>
+      <c r="C14" s="16">
+        <f>SUM(C5:C13)</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B15" s="16">
-        <f>SUM(B5:B14)</f>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Research: conferences</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>COUNTIF('Research papers'!$B$5:$B$51,"Conference")</f>
         <v/>
       </c>
-      <c r="C15" s="16">
-        <f>SUM(C5:C14)</f>
+      <c r="C16" s="15">
+        <f>COUNTIFS('Research papers'!$B$5:$B$51,"Conference",'Research papers'!$A$5:$A$51,"Yes")</f>
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Research: journals</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>COUNTIF('Research papers'!$B$5:$B$51,"Journal")</f>
+        <v/>
+      </c>
+      <c r="C17" s="15">
+        <f>COUNTIFS('Research papers'!$B$5:$B$51,"Journal",'Research papers'!$A$5:$A$51,"Yes")</f>
+        <v/>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Research: arXiv topics</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>COUNTIF('Research papers'!$B$5:$B$51,"Topic search")</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>COUNTIFS('Research papers'!$B$5:$B$51,"Topic search",'Research papers'!$A$5:$A$51,"Yes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Anthropic, Meta AI (ai.meta.com) and The Batch (DeepLearning.AI) publish no RSS feed, so they can't be followed automatically. Their stories still show up through Techmeme, The Verge, The Decoder and others.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Anthropic publishes no RSS feed, so its news, engineering and research pages are read directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>IEA: only its reports are shown, each linked straight to the report on iea.org (found through Google News, because the IEA blocks automated access).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>arXiv searches are tuned to your research (agents, AI for SE, LLM energy, uncertainty). Tell me other keywords and I'll add them.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Any YouTube channel can be added: give me the channel link.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>The site updates itself every hour: new posts from every chosen source appear on their own.</t>
         </is>
@@ -6566,11 +5855,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
My Radar: add Software engineering for AI (SE4AI) next to AI for SE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tech-Pulse-Sources.xlsx
+++ b/Tech-Pulse-Sources.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$4:$I$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Research papers'!$A$4:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Research papers'!$A$4:$G$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4065,7 +4065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5442,17 +5442,17 @@
       <c r="C41" s="5" t="inlineStr"/>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Green AI &amp; energy</t>
+          <t>Software engineering for AI</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>(abs:"energy consumption" OR abs:"energy efficiency" OR abs:"carbon footprint" OR abs:"green software") AND (abs:LLM OR abs:"language model" OR abs:software)</t>
+          <t>cat:cs.SE AND (abs:"AI systems" OR abs:"AI-based systems" OR abs:"AI-enabled systems" OR abs:"ML systems" OR abs:"machine learning systems" OR abs:"deep learning systems" OR abs:"LLM-based systems" OR abs:"LLM-based applications" OR abs:"LLM applications" OR abs:"agentic systems" OR abs:"compound AI" OR abs:MLOps OR abs:LLMOps OR abs:"AI engineering" OR abs:SE4AI)</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>16 in last 10 days</t>
+          <t>0 in last 10 days</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -5475,17 +5475,17 @@
       <c r="C42" s="5" t="inlineStr"/>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Uncertainty in LLMs &amp; agents</t>
+          <t>Green AI &amp; energy</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>abs:uncertainty AND (abs:LLM OR abs:agent)</t>
+          <t>(abs:"energy consumption" OR abs:"energy efficiency" OR abs:"carbon footprint" OR abs:"green software") AND (abs:LLM OR abs:"language model" OR abs:software)</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>50 in last 10 days</t>
+          <t>16 in last 10 days</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -5508,35 +5508,65 @@
       <c r="C43" s="5" t="inlineStr"/>
       <c r="D43" s="5" t="inlineStr">
         <is>
+          <t>Uncertainty in LLMs &amp; agents</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>abs:uncertainty AND (abs:LLM OR abs:agent)</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>50 in last 10 days</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>arXiv search</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Topic search</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
           <t>Every new cs.SE paper</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>cat:cs.SE</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>60 in last 10 days</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>arXiv search</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="13" t="n"/>
-      <c r="D44" s="11" t="inlineStr">
-        <is>
-          <t>(add your own here)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="n"/>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>(add your own here)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="n"/>
@@ -5556,18 +5586,21 @@
     <row r="51">
       <c r="A51" s="13" t="n"/>
     </row>
+    <row r="52">
+      <c r="A52" s="13" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G51"/>
+  <autoFilter ref="A4:G52"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G51">
+  <conditionalFormatting sqref="A5:G52">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$A5="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5:A51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A5:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5780,11 +5813,11 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>COUNTIF('Research papers'!$B$5:$B$51,"Conference")</f>
+        <f>COUNTIF('Research papers'!$B$5:$B$52,"Conference")</f>
         <v/>
       </c>
       <c r="C16" s="15">
-        <f>COUNTIFS('Research papers'!$B$5:$B$51,"Conference",'Research papers'!$A$5:$A$51,"Yes")</f>
+        <f>COUNTIFS('Research papers'!$B$5:$B$52,"Conference",'Research papers'!$A$5:$A$52,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -5795,11 +5828,11 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>COUNTIF('Research papers'!$B$5:$B$51,"Journal")</f>
+        <f>COUNTIF('Research papers'!$B$5:$B$52,"Journal")</f>
         <v/>
       </c>
       <c r="C17" s="15">
-        <f>COUNTIFS('Research papers'!$B$5:$B$51,"Journal",'Research papers'!$A$5:$A$51,"Yes")</f>
+        <f>COUNTIFS('Research papers'!$B$5:$B$52,"Journal",'Research papers'!$A$5:$A$52,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -5810,11 +5843,11 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>COUNTIF('Research papers'!$B$5:$B$51,"Topic search")</f>
+        <f>COUNTIF('Research papers'!$B$5:$B$52,"Topic search")</f>
         <v/>
       </c>
       <c r="C18" s="15">
-        <f>COUNTIFS('Research papers'!$B$5:$B$51,"Topic search",'Research papers'!$A$5:$A$51,"Yes")</f>
+        <f>COUNTIFS('Research papers'!$B$5:$B$52,"Topic search",'Research papers'!$A$5:$A$52,"Yes")</f>
         <v/>
       </c>
     </row>

</xml_diff>